<commit_message>
Corrige tamaños de fotos, agrega split Anterior/Actual y fija la barra lateral
</commit_message>
<xml_diff>
--- a/public/plantillas/DR000_12501191.xlsx
+++ b/public/plantillas/DR000_12501191.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Imágenes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">DR!$B$1:$N$97</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">DR!$B$1:$N$98</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Imágenes!$B$1:$N$93</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -2909,7 +2909,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:N98"/>
+  <dimension ref="B1:N99"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="4.28515625" style="4" customWidth="1"/>
@@ -4447,7 +4447,7 @@
         <v>1</v>
       </c>
       <c r="G64" s="70">
-        <f>11*E64</f>
+        <f>$J$9*E64</f>
         <v>0</v>
       </c>
       <c r="I64" s="134" t="s">
@@ -4480,7 +4480,7 @@
         <v>1</v>
       </c>
       <c r="G65" s="70">
-        <f t="shared" ref="G65:G75" si="10">11*E65</f>
+        <f t="shared" ref="G65:G75" si="10">$J$9*E65</f>
         <v>0</v>
       </c>
       <c r="I65" s="134" t="s">
@@ -4574,8 +4574,10 @@
       <c r="N68" s="6"/>
     </row>
     <row r="69" spans="2:14">
-      <c r="B69" s="147" t="s">
-        <v>97</v>
+      <c r="B69" s="147" t="inlineStr">
+        <is>
+          <t>Asesor Prevencion de Riesgos</t>
+        </is>
       </c>
       <c r="C69" s="148"/>
       <c r="D69" s="74">
@@ -4785,24 +4787,30 @@
       </c>
     </row>
     <row r="80" spans="2:14" ht="15" thickBot="1">
-      <c r="B80" s="134" t="s">
-        <v>106</v>
+      <c r="B80" s="134" t="inlineStr">
+        <is>
+          <t>Total HH Directas Acumuladas Anterior</t>
+        </is>
       </c>
       <c r="C80" s="135"/>
       <c r="D80" s="139">
         <v>0</v>
       </c>
       <c r="E80" s="140"/>
-      <c r="F80" s="134" t="s">
-        <v>107</v>
+      <c r="F80" s="134" t="inlineStr">
+        <is>
+          <t>Total HM Acumuladas Anterior</t>
+        </is>
       </c>
       <c r="G80" s="138"/>
       <c r="H80" s="135"/>
       <c r="I80" s="98">
         <v>0</v>
       </c>
-      <c r="J80" s="134" t="s">
-        <v>108</v>
+      <c r="J80" s="134" t="inlineStr">
+        <is>
+          <t>Total HH Indirectas Acumuladas Anterior</t>
+        </is>
       </c>
       <c r="K80" s="138"/>
       <c r="L80" s="138"/>
@@ -4811,62 +4819,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:14" ht="15" customHeight="1" thickBot="1">
-      <c r="B81" s="5"/>
-      <c r="N81" s="6"/>
+    <row r="81" spans="2:14" ht="15" thickBot="1">
+      <c r="B81" s="134" t="inlineStr">
+        <is>
+          <t>Total HH Directas Acumuladas Actual</t>
+        </is>
+      </c>
+      <c r="C81" s="135"/>
+      <c r="D81" s="139">
+        <f>D79+D80</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="140"/>
+      <c r="F81" s="134" t="inlineStr">
+        <is>
+          <t>Total HM Acumuladas Actual</t>
+        </is>
+      </c>
+      <c r="G81" s="138"/>
+      <c r="H81" s="135"/>
+      <c r="I81" s="98">
+        <f>I79+I80</f>
+        <v>0</v>
+      </c>
+      <c r="J81" s="134" t="inlineStr">
+        <is>
+          <t>Total HH Indirectas Acumuladas Actual</t>
+        </is>
+      </c>
+      <c r="K81" s="138"/>
+      <c r="L81" s="138"/>
+      <c r="M81" s="135"/>
+      <c r="N81" s="98">
+        <f>N79+N80</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="82" spans="2:14" ht="15" customHeight="1" thickBot="1">
-      <c r="B82" s="126" t="s">
+      <c r="B82" s="5"/>
+      <c r="N82" s="6"/>
+    </row>
+    <row r="83" spans="2:14" ht="15" customHeight="1" thickBot="1">
+      <c r="B83" s="126" t="s">
         <v>109</v>
       </c>
-      <c r="C82" s="127"/>
-      <c r="D82" s="127" t="s">
+      <c r="C83" s="127"/>
+      <c r="D83" s="127" t="s">
         <v>110</v>
       </c>
-      <c r="E82" s="127"/>
-      <c r="F82" s="127"/>
-      <c r="G82" s="127"/>
-      <c r="H82" s="127"/>
-      <c r="I82" s="127"/>
-      <c r="J82" s="127"/>
-      <c r="K82" s="127"/>
-      <c r="L82" s="127"/>
-      <c r="M82" s="127"/>
-      <c r="N82" s="128"/>
-    </row>
-    <row r="83" spans="2:14" ht="14.45" customHeight="1">
-      <c r="B83" s="129"/>
-      <c r="C83" s="130"/>
-      <c r="D83" s="141"/>
-      <c r="E83" s="142"/>
-      <c r="F83" s="142"/>
-      <c r="G83" s="142"/>
-      <c r="H83" s="142"/>
-      <c r="I83" s="142"/>
-      <c r="J83" s="142"/>
-      <c r="K83" s="142"/>
-      <c r="L83" s="142"/>
-      <c r="M83" s="142"/>
-      <c r="N83" s="143"/>
-    </row>
-    <row r="84" spans="2:14">
-      <c r="B84" s="144"/>
-      <c r="C84" s="145"/>
-      <c r="D84" s="120"/>
-      <c r="E84" s="121"/>
-      <c r="F84" s="121"/>
-      <c r="G84" s="121"/>
-      <c r="H84" s="121"/>
-      <c r="I84" s="121"/>
-      <c r="J84" s="121"/>
-      <c r="K84" s="121"/>
-      <c r="L84" s="121"/>
-      <c r="M84" s="121"/>
-      <c r="N84" s="122"/>
+      <c r="E83" s="127"/>
+      <c r="F83" s="127"/>
+      <c r="G83" s="127"/>
+      <c r="H83" s="127"/>
+      <c r="I83" s="127"/>
+      <c r="J83" s="127"/>
+      <c r="K83" s="127"/>
+      <c r="L83" s="127"/>
+      <c r="M83" s="127"/>
+      <c r="N83" s="128"/>
+    </row>
+    <row r="84" spans="2:14" ht="14.45" customHeight="1">
+      <c r="B84" s="129"/>
+      <c r="C84" s="130"/>
+      <c r="D84" s="141"/>
+      <c r="E84" s="142"/>
+      <c r="F84" s="142"/>
+      <c r="G84" s="142"/>
+      <c r="H84" s="142"/>
+      <c r="I84" s="142"/>
+      <c r="J84" s="142"/>
+      <c r="K84" s="142"/>
+      <c r="L84" s="142"/>
+      <c r="M84" s="142"/>
+      <c r="N84" s="143"/>
     </row>
     <row r="85" spans="2:14">
-      <c r="B85" s="209"/>
-      <c r="C85" s="210"/>
+      <c r="B85" s="144"/>
+      <c r="C85" s="145"/>
       <c r="D85" s="120"/>
       <c r="E85" s="121"/>
       <c r="F85" s="121"/>
@@ -4879,69 +4908,69 @@
       <c r="M85" s="121"/>
       <c r="N85" s="122"/>
     </row>
-    <row r="86" spans="2:14" ht="15" thickBot="1">
-      <c r="B86" s="211"/>
-      <c r="C86" s="212"/>
-      <c r="D86" s="123"/>
-      <c r="E86" s="124"/>
-      <c r="F86" s="124"/>
-      <c r="G86" s="124"/>
-      <c r="H86" s="124"/>
-      <c r="I86" s="124"/>
-      <c r="J86" s="124"/>
-      <c r="K86" s="124"/>
-      <c r="L86" s="124"/>
-      <c r="M86" s="124"/>
-      <c r="N86" s="125"/>
-    </row>
-    <row r="87" spans="2:14" ht="15.75" thickBot="1">
-      <c r="B87" s="126" t="s">
+    <row r="86" spans="2:14">
+      <c r="B86" s="209"/>
+      <c r="C86" s="210"/>
+      <c r="D86" s="120"/>
+      <c r="E86" s="121"/>
+      <c r="F86" s="121"/>
+      <c r="G86" s="121"/>
+      <c r="H86" s="121"/>
+      <c r="I86" s="121"/>
+      <c r="J86" s="121"/>
+      <c r="K86" s="121"/>
+      <c r="L86" s="121"/>
+      <c r="M86" s="121"/>
+      <c r="N86" s="122"/>
+    </row>
+    <row r="87" spans="2:14" ht="15" thickBot="1">
+      <c r="B87" s="211"/>
+      <c r="C87" s="212"/>
+      <c r="D87" s="123"/>
+      <c r="E87" s="124"/>
+      <c r="F87" s="124"/>
+      <c r="G87" s="124"/>
+      <c r="H87" s="124"/>
+      <c r="I87" s="124"/>
+      <c r="J87" s="124"/>
+      <c r="K87" s="124"/>
+      <c r="L87" s="124"/>
+      <c r="M87" s="124"/>
+      <c r="N87" s="125"/>
+    </row>
+    <row r="88" spans="2:14" ht="15.75" thickBot="1">
+      <c r="B88" s="126" t="s">
         <v>109</v>
       </c>
-      <c r="C87" s="127"/>
-      <c r="D87" s="127" t="s">
+      <c r="C88" s="127"/>
+      <c r="D88" s="127" t="s">
         <v>111</v>
       </c>
-      <c r="E87" s="127"/>
-      <c r="F87" s="127"/>
-      <c r="G87" s="127"/>
-      <c r="H87" s="127"/>
-      <c r="I87" s="127"/>
-      <c r="J87" s="127"/>
-      <c r="K87" s="127"/>
-      <c r="L87" s="127"/>
-      <c r="M87" s="127"/>
-      <c r="N87" s="128"/>
-    </row>
-    <row r="88" spans="2:14" ht="14.45" customHeight="1">
-      <c r="B88" s="129"/>
-      <c r="C88" s="130"/>
-      <c r="D88" s="131"/>
-      <c r="E88" s="132"/>
-      <c r="F88" s="132"/>
-      <c r="G88" s="132"/>
-      <c r="H88" s="132"/>
-      <c r="I88" s="132"/>
-      <c r="J88" s="132"/>
-      <c r="K88" s="132"/>
-      <c r="L88" s="132"/>
-      <c r="M88" s="132"/>
-      <c r="N88" s="133"/>
-    </row>
-    <row r="89" spans="2:14">
-      <c r="B89" s="39"/>
-      <c r="C89" s="19"/>
-      <c r="D89" s="120"/>
-      <c r="E89" s="121"/>
-      <c r="F89" s="121"/>
-      <c r="G89" s="121"/>
-      <c r="H89" s="121"/>
-      <c r="I89" s="121"/>
-      <c r="J89" s="121"/>
-      <c r="K89" s="121"/>
-      <c r="L89" s="121"/>
-      <c r="M89" s="121"/>
-      <c r="N89" s="122"/>
+      <c r="E88" s="127"/>
+      <c r="F88" s="127"/>
+      <c r="G88" s="127"/>
+      <c r="H88" s="127"/>
+      <c r="I88" s="127"/>
+      <c r="J88" s="127"/>
+      <c r="K88" s="127"/>
+      <c r="L88" s="127"/>
+      <c r="M88" s="127"/>
+      <c r="N88" s="128"/>
+    </row>
+    <row r="89" spans="2:14" ht="14.45" customHeight="1">
+      <c r="B89" s="129"/>
+      <c r="C89" s="130"/>
+      <c r="D89" s="131"/>
+      <c r="E89" s="132"/>
+      <c r="F89" s="132"/>
+      <c r="G89" s="132"/>
+      <c r="H89" s="132"/>
+      <c r="I89" s="132"/>
+      <c r="J89" s="132"/>
+      <c r="K89" s="132"/>
+      <c r="L89" s="132"/>
+      <c r="M89" s="132"/>
+      <c r="N89" s="133"/>
     </row>
     <row r="90" spans="2:14">
       <c r="B90" s="39"/>
@@ -4958,142 +4987,157 @@
       <c r="M90" s="121"/>
       <c r="N90" s="122"/>
     </row>
-    <row r="91" spans="2:14" ht="15" customHeight="1" thickBot="1">
-      <c r="B91" s="40"/>
-      <c r="C91" s="41"/>
-      <c r="D91" s="123"/>
-      <c r="E91" s="124"/>
-      <c r="F91" s="124"/>
-      <c r="G91" s="124"/>
-      <c r="H91" s="124"/>
-      <c r="I91" s="124"/>
-      <c r="J91" s="124"/>
-      <c r="K91" s="124"/>
-      <c r="L91" s="124"/>
-      <c r="M91" s="124"/>
-      <c r="N91" s="125"/>
-    </row>
-    <row r="92" spans="2:14" ht="15" thickBot="1">
-      <c r="B92" s="42"/>
-      <c r="C92" s="43"/>
-      <c r="D92" s="43"/>
-      <c r="E92" s="43"/>
-      <c r="N92" s="6"/>
-    </row>
-    <row r="93" spans="2:14" ht="15" customHeight="1" thickBot="1">
-      <c r="B93" s="114" t="s">
+    <row r="91" spans="2:14">
+      <c r="B91" s="39"/>
+      <c r="C91" s="19"/>
+      <c r="D91" s="120"/>
+      <c r="E91" s="121"/>
+      <c r="F91" s="121"/>
+      <c r="G91" s="121"/>
+      <c r="H91" s="121"/>
+      <c r="I91" s="121"/>
+      <c r="J91" s="121"/>
+      <c r="K91" s="121"/>
+      <c r="L91" s="121"/>
+      <c r="M91" s="121"/>
+      <c r="N91" s="122"/>
+    </row>
+    <row r="92" spans="2:14" ht="15" customHeight="1" thickBot="1">
+      <c r="B92" s="40"/>
+      <c r="C92" s="41"/>
+      <c r="D92" s="123"/>
+      <c r="E92" s="124"/>
+      <c r="F92" s="124"/>
+      <c r="G92" s="124"/>
+      <c r="H92" s="124"/>
+      <c r="I92" s="124"/>
+      <c r="J92" s="124"/>
+      <c r="K92" s="124"/>
+      <c r="L92" s="124"/>
+      <c r="M92" s="124"/>
+      <c r="N92" s="125"/>
+    </row>
+    <row r="93" spans="2:14" ht="15" thickBot="1">
+      <c r="B93" s="42"/>
+      <c r="C93" s="43"/>
+      <c r="D93" s="43"/>
+      <c r="E93" s="43"/>
+      <c r="N93" s="6"/>
+    </row>
+    <row r="94" spans="2:14" ht="15" customHeight="1" thickBot="1">
+      <c r="B94" s="114" t="s">
         <v>112</v>
       </c>
-      <c r="C93" s="115"/>
-      <c r="D93" s="115"/>
-      <c r="E93" s="116"/>
-      <c r="F93" s="117" t="s">
+      <c r="C94" s="115"/>
+      <c r="D94" s="115"/>
+      <c r="E94" s="116"/>
+      <c r="F94" s="117" t="s">
         <v>113</v>
       </c>
-      <c r="G93" s="118"/>
-      <c r="H93" s="118"/>
-      <c r="I93" s="119"/>
-      <c r="J93" s="117" t="s">
+      <c r="G94" s="118"/>
+      <c r="H94" s="118"/>
+      <c r="I94" s="119"/>
+      <c r="J94" s="117" t="s">
         <v>114</v>
       </c>
-      <c r="K93" s="118"/>
-      <c r="L93" s="118"/>
-      <c r="M93" s="118"/>
-      <c r="N93" s="119"/>
-    </row>
-    <row r="94" spans="2:14" ht="34.15" customHeight="1">
-      <c r="B94" s="44" t="s">
+      <c r="K94" s="118"/>
+      <c r="L94" s="118"/>
+      <c r="M94" s="118"/>
+      <c r="N94" s="119"/>
+    </row>
+    <row r="95" spans="2:14" ht="34.15" customHeight="1">
+      <c r="B95" s="44" t="s">
         <v>115</v>
       </c>
-      <c r="C94" s="60" t="s">
+      <c r="C95" s="60" t="s">
         <v>116</v>
       </c>
-      <c r="D94" s="45"/>
-      <c r="E94" s="46"/>
-      <c r="F94" s="47" t="s">
+      <c r="D95" s="45"/>
+      <c r="E95" s="46"/>
+      <c r="F95" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="G94" s="45" t="s">
+      <c r="G95" s="45" t="s">
         <v>118</v>
       </c>
-      <c r="H94" s="45"/>
-      <c r="I94" s="46"/>
-      <c r="J94" s="47" t="s">
+      <c r="H95" s="45"/>
+      <c r="I95" s="46"/>
+      <c r="J95" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="K94" s="45"/>
-      <c r="L94" s="45"/>
-      <c r="M94" s="45"/>
-      <c r="N94" s="6"/>
-    </row>
-    <row r="95" spans="2:14" ht="33.6" customHeight="1">
-      <c r="B95" s="48" t="s">
+      <c r="K95" s="45"/>
+      <c r="L95" s="45"/>
+      <c r="M95" s="45"/>
+      <c r="N95" s="6"/>
+    </row>
+    <row r="96" spans="2:14" ht="33.6" customHeight="1">
+      <c r="B96" s="48" t="s">
         <v>119</v>
       </c>
-      <c r="C95" s="49"/>
-      <c r="D95" s="49"/>
-      <c r="E95" s="50"/>
-      <c r="F95" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="G95" s="49"/>
-      <c r="H95" s="49"/>
-      <c r="I95" s="50"/>
-      <c r="J95" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="K95" s="49"/>
-      <c r="L95" s="49"/>
-      <c r="M95" s="49"/>
-      <c r="N95" s="6"/>
-    </row>
-    <row r="96" spans="2:14" ht="35.450000000000003" customHeight="1">
-      <c r="B96" s="48" t="s">
-        <v>120</v>
-      </c>
-      <c r="C96" s="61">
-        <f>J5</f>
-        <v>0</v>
-      </c>
-      <c r="D96" s="52"/>
+      <c r="C96" s="49"/>
+      <c r="D96" s="49"/>
       <c r="E96" s="50"/>
       <c r="F96" s="51" t="s">
-        <v>121</v>
-      </c>
-      <c r="G96" s="61">
-        <f>C96</f>
-        <v>0</v>
-      </c>
-      <c r="H96" s="52"/>
+        <v>119</v>
+      </c>
+      <c r="G96" s="49"/>
+      <c r="H96" s="49"/>
       <c r="I96" s="50"/>
       <c r="J96" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="K96" s="49"/>
+      <c r="L96" s="49"/>
+      <c r="M96" s="49"/>
+      <c r="N96" s="6"/>
+    </row>
+    <row r="97" spans="2:14" ht="35.450000000000003" customHeight="1">
+      <c r="B97" s="48" t="s">
+        <v>120</v>
+      </c>
+      <c r="C97" s="61">
+        <f>J5</f>
+        <v>0</v>
+      </c>
+      <c r="D97" s="52"/>
+      <c r="E97" s="50"/>
+      <c r="F97" s="51" t="s">
         <v>121</v>
       </c>
-      <c r="K96" s="52"/>
-      <c r="L96" s="52"/>
-      <c r="M96" s="52"/>
-      <c r="N96" s="6"/>
-    </row>
-    <row r="97" spans="2:14" ht="15" customHeight="1" thickBot="1">
-      <c r="B97" s="53"/>
-      <c r="C97" s="54"/>
-      <c r="D97" s="54"/>
-      <c r="E97" s="55"/>
-      <c r="F97" s="56"/>
-      <c r="G97" s="57"/>
-      <c r="H97" s="57"/>
-      <c r="I97" s="55"/>
-      <c r="J97" s="56"/>
-      <c r="K97" s="57"/>
-      <c r="L97" s="57"/>
-      <c r="M97" s="57"/>
-      <c r="N97" s="13"/>
-    </row>
-    <row r="98" spans="2:14">
-      <c r="B98" s="2"/>
+      <c r="G97" s="61">
+        <f>C97</f>
+        <v>0</v>
+      </c>
+      <c r="H97" s="52"/>
+      <c r="I97" s="50"/>
+      <c r="J97" s="51" t="s">
+        <v>121</v>
+      </c>
+      <c r="K97" s="52"/>
+      <c r="L97" s="52"/>
+      <c r="M97" s="52"/>
+      <c r="N97" s="6"/>
+    </row>
+    <row r="98" spans="2:14" ht="15" customHeight="1" thickBot="1">
+      <c r="B98" s="53"/>
+      <c r="C98" s="54"/>
+      <c r="D98" s="54"/>
+      <c r="E98" s="55"/>
+      <c r="F98" s="56"/>
+      <c r="G98" s="57"/>
+      <c r="H98" s="57"/>
+      <c r="I98" s="55"/>
+      <c r="J98" s="56"/>
+      <c r="K98" s="57"/>
+      <c r="L98" s="57"/>
+      <c r="M98" s="57"/>
+      <c r="N98" s="13"/>
+    </row>
+    <row r="99" spans="2:14">
+      <c r="B99" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="100">
+  <mergeCells count="104">
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="K10:N10"/>
@@ -5166,12 +5210,12 @@
     <mergeCell ref="B68:C68"/>
     <mergeCell ref="B69:C69"/>
     <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="D82:N82"/>
     <mergeCell ref="B83:C83"/>
     <mergeCell ref="D83:N83"/>
     <mergeCell ref="B84:C84"/>
     <mergeCell ref="D84:N84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="D85:N85"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="D79:E79"/>
     <mergeCell ref="F79:H79"/>
@@ -5180,20 +5224,24 @@
     <mergeCell ref="D80:E80"/>
     <mergeCell ref="F80:H80"/>
     <mergeCell ref="J80:M80"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="F93:I93"/>
-    <mergeCell ref="J93:N93"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="D85:N85"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="F94:I94"/>
+    <mergeCell ref="J94:N94"/>
     <mergeCell ref="B86:C86"/>
     <mergeCell ref="D86:N86"/>
     <mergeCell ref="B87:C87"/>
     <mergeCell ref="D87:N87"/>
     <mergeCell ref="B88:C88"/>
     <mergeCell ref="D88:N88"/>
+    <mergeCell ref="B89:C89"/>
     <mergeCell ref="D89:N89"/>
     <mergeCell ref="D90:N90"/>
     <mergeCell ref="D91:N91"/>
+    <mergeCell ref="D92:N92"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="F81:H81"/>
+    <mergeCell ref="J81:M81"/>
   </mergeCells>
   <pageMargins left="1.1023622047244095" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="45" orientation="portrait" r:id="rId1"/>
@@ -6547,7 +6595,7 @@
         <v>115</v>
       </c>
       <c r="C90" s="60" t="str">
-        <f>+DR!C94</f>
+        <f>+DR!C95</f>
         <v>Ericson Ramirez</v>
       </c>
       <c r="D90" s="45"/>
@@ -6556,7 +6604,7 @@
         <v>117</v>
       </c>
       <c r="G90" s="45" t="str">
-        <f>+DR!G94</f>
+        <f>+DR!G95</f>
         <v>Sara Cofré</v>
       </c>
       <c r="H90" s="45"/>
@@ -6595,7 +6643,7 @@
         <v>120</v>
       </c>
       <c r="C92" s="61">
-        <f>+DR!C96</f>
+        <f>+DR!C97</f>
         <v>0</v>
       </c>
       <c r="D92" s="52"/>

</xml_diff>

<commit_message>
Corrige el ancho distinto de las fotos en la hoja Imágenes del Excel
Las columnas B..N de la hoja "Imágenes" tenían anchos muy distintos entre
sí (B=27.3, F/M/N=11.6 por ejemplo). La grilla de fotos reparte esas
columnas en 3 franjas iguales por ÍNDICE de columna (4 columnas cada
una), pero como los anchos reales no eran uniformes, cada franja
terminaba con un ancho en píxeles distinto — la tarjeta de la izquierda
(que incluye la columna B, la más ancha) salía visiblemente más ancha
que la de la derecha, tal como se ve en captura real de Excel.

Se iguala el ancho de las 13 columnas (B..N) a un único valor (promedio
de los anchos originales, para no cambiar mucho el ancho total de la
hoja), así las 3 franjas de la grilla quedan con el mismo ancho real.
Esto es independiente del fix anterior de aspect-ratio/altura — eran dos
causas distintas del mismo síntoma general ("las fotos salen de tamaños
distintos").
</commit_message>
<xml_diff>
--- a/public/plantillas/DR000_12501191.xlsx
+++ b/public/plantillas/DR000_12501191.xlsx
@@ -5258,16 +5258,7 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="8.28515625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="4" customWidth="1"/>
-    <col min="5" max="6" width="11.5703125" style="4"/>
-    <col min="7" max="7" width="16.42578125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" style="4" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" style="4"/>
-    <col min="11" max="11" width="12.140625" style="4" customWidth="1"/>
-    <col min="12" max="14" width="11.5703125" style="4"/>
+    <col min="2" max="14" width="13.668870192307692" style="4" customWidth="1"/>
     <col min="15" max="15" width="5.85546875" style="4" customWidth="1"/>
     <col min="16" max="16384" width="11.5703125" style="4"/>
   </cols>

</xml_diff>